<commit_message>
Correction qualité FSH : extensions, exemples et aliases
- MesOriginalData.fsh : correction du ^short copié-collé ("Nombre de jours" → "Valeur originale de la donnée")
- aliases.fsh : centralisation des aliases $loinc, $observation-category, $ContinuaDeviceIdentifiers
- ObservationHb1AcExample.fsh : suppression de la méthode référençant un ValueSet comme CodeSystem
- Renommage des fichiers d'exemples selon la convention *Example.fsh
- sushi-config.yaml : correction du libellé de juridiction ("France" → "France (la)")

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> d4e2e1fc5022167911d98f8c32e1929b27740f7d
</commit_message>
<xml_diff>
--- a/nr-fix/ig/StructureDefinition-mesures-bundle-flux-alimentation-biologie.xlsx
+++ b/nr-fix/ig/StructureDefinition-mesures-bundle-flux-alimentation-biologie.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-31T09:05:32+00:00</t>
+    <t>2026-03-31T09:17:37+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -75,7 +75,7 @@
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t>France</t>
+    <t>France (la)</t>
   </si>
   <si>
     <t>Description</t>

</xml_diff>